<commit_message>
fix entry items tags and lists
</commit_message>
<xml_diff>
--- a/data/swisscom_bedag_stadt-zh.xlsx
+++ b/data/swisscom_bedag_stadt-zh.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,22 +461,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Opportunity x</t>
+          <t>TEst</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Less Than 1 Year</t>
+          <t>Ready</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Automation</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>New</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -491,6 +491,74 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Test 2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Less Than 1 Year</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;br&gt;&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Test Tags</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>On Track</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;br&gt;&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix save on change
</commit_message>
<xml_diff>
--- a/data/swisscom_bedag_stadt-zh.xlsx
+++ b/data/swisscom_bedag_stadt-zh.xlsx
@@ -505,7 +505,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>auto</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -515,21 +515,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>&lt;p&gt;&lt;br&gt;&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+          <t>&lt;p&gt;check&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Test Tags</t>
+          <t>Test Tags!</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -539,7 +535,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Auto</t>
+          <t>auto</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -552,11 +548,7 @@
           <t>&lt;p&gt;&lt;br&gt;&lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
     </row>

</xml_diff>